<commit_message>
Handle more logic to improve correctness
</commit_message>
<xml_diff>
--- a/data/Mar/Data-import.xlsx
+++ b/data/Mar/Data-import.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Mar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92681E77-7BB5-47CB-94E9-C6E34A755286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EC96FD5-AFB6-46F2-BF20-6B6CB16D93CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{07C974F8-99FB-4C7E-9A60-2AB7B39D2515}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6008" uniqueCount="1998">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6018" uniqueCount="2002">
   <si>
     <t>THU 2</t>
   </si>
@@ -6050,13 +6050,25 @@
   </si>
   <si>
     <t>137/31/14 phan anh phường bình trị đông</t>
+  </si>
+  <si>
+    <t>Ms Thuyền Tố Như ari</t>
+  </si>
+  <si>
+    <t>HD010485</t>
+  </si>
+  <si>
+    <t>C16-17 lô C1, đường DD5, phường Tân Hưng Thuận</t>
+  </si>
+  <si>
+    <t>13-04-2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6091,6 +6103,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="14">
@@ -6198,7 +6216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -6288,6 +6306,9 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -26846,7 +26867,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:S40"/>
+  <dimension ref="A1:S41"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" style="13" customWidth="1"/>
@@ -28621,6 +28642,56 @@
         <v>443</v>
       </c>
       <c r="Q40" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" s="57" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="55"/>
+      <c r="B41" s="55" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="55" t="s">
+        <v>1998</v>
+      </c>
+      <c r="D41" s="55" t="s">
+        <v>1999</v>
+      </c>
+      <c r="E41" s="55" t="s">
+        <v>2000</v>
+      </c>
+      <c r="F41" s="56">
+        <v>12</v>
+      </c>
+      <c r="G41" s="56">
+        <v>870</v>
+      </c>
+      <c r="H41" s="56">
+        <v>0</v>
+      </c>
+      <c r="I41" s="56">
+        <f>G41-H41</f>
+        <v>870</v>
+      </c>
+      <c r="J41" s="55" t="s">
+        <v>425</v>
+      </c>
+      <c r="K41" s="55" t="s">
+        <v>22</v>
+      </c>
+      <c r="L41" s="55" t="s">
+        <v>2001</v>
+      </c>
+      <c r="M41" s="55"/>
+      <c r="N41" s="55" t="s">
+        <v>275</v>
+      </c>
+      <c r="O41" s="55" t="s">
+        <v>275</v>
+      </c>
+      <c r="P41" s="55" t="s">
+        <v>427</v>
+      </c>
+      <c r="Q41" s="57">
         <v>1</v>
       </c>
     </row>

</xml_diff>